<commit_message>
Docs: LIS2DW12 address 0x19 (SA0 high) in architecture, pin list and BOM design changes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Schematics/RevA/BOM/Jot_RevA_BOM.xlsx
+++ b/Schematics/RevA/BOM/Jot_RevA_BOM.xlsx
@@ -2477,7 +2477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2689,6 +2689,23 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Accelerometer address: LIS2DW12 0x18 (SA0 low) -&gt; 0x19 (SA0 high)</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>SDO/SA0 has an internal pull-up (about 22 kOhm at 3.3 V, datasheet Table 3) that, unlike CS, cannot be disconnected in a register. Tied to GND it would draw about 150 uA all the time, about 20x the board sleep budget.</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>U7 SDO/SA0 and CS tied to +3V3. Firmware uses I2C address 0x19. Changed 2026-10-04.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Draft 3 RGB LED in BOM and pin list: common-anode TJ-S1615SW6TGLCCYRGB-A5 on +BATT, Q3-Q5 AO3400A, R15-R17 pull-downs, R9/R10 560R; datasheet added
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Schematics/RevA/BOM/Jot_RevA_BOM.xlsx
+++ b/Schematics/RevA/BOM/Jot_RevA_BOM.xlsx
@@ -797,7 +797,7 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
@@ -816,12 +816,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Q1,Q3,Q4,Q5</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>N-MOSFET, buzzer driver, SOT-23</t>
+          <t>N-MOSFET, SOT-23: buzzer driver (Q1) and RGB LED cathode switches (Q3-Q5)</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>TJ-S1615SW6TGLCCSRGB-A5</t>
+          <t>TJ-S1615SW6TGLCCYRGB-A5</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1051,7 +1051,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>C273611</t>
+          <t>C273610</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1061,7 +1061,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>RGB LED common cathode, 1.6x1.5 mm</t>
+          <t>RGB LED common anode, 1.6x1.5 mm (pin 1 anode; 2 B, 3 G, 4 R cathodes)</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>0402WGF1000TCE</t>
+          <t>0402WGF5600TCE</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1255,7 +1255,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>100R 1% 0402 (RGB green, blue)</t>
+          <t>560R 1% 0402 (RGB green, blue)</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1291,7 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
@@ -1310,12 +1310,12 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>R12,R13</t>
+          <t>R12,R13,R15,R16,R17</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>100k 1% 0402 (Q1 gate pull-down, Q2 gate pull-up)</t>
+          <t>100k 1% 0402 (Q1, Q3, Q4, Q5 gate pull-downs; Q2 gate pull-up)</t>
         </is>
       </c>
     </row>
@@ -1785,7 +1785,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Q1, Q3-Q5</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -1805,7 +1805,7 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Replaces 2N7002: buzzer can draw ~100 mA and 2N7002 is only rated 115 mA with 2.5 V threshold. AO3400A is logic-level.</t>
+          <t>Replaces 2N7002: buzzer can draw ~100 mA and 2N7002 is only rated 115 mA with 2.5 V threshold. AO3400A is logic-level. Draft 3: the same part switches the RGB LED cathodes (Q3-Q5), gate from a 3.3 V GPIO with a 100k pull-down.</t>
         </is>
       </c>
     </row>
@@ -2060,22 +2060,22 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>TJ-S1615SW6TGLCCSRGB-A5</t>
+          <t>TJ-S1615SW6TGLCCYRGB-A5</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>C273611</t>
+          <t>C273610</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Verified exists - check stock</t>
+          <t>Verified - datasheet read</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Common CATHODE (changed from common anode): each color driven high from a GPIO. Blue/green Vf 2.8-3.6 V, so dimmer at 3.3 V - fine for a status LED.</t>
+          <t>Common ANODE (draft 3). Datasheet (Datasheets/UI/TJ-S1615SW6TGLCCYRGB-A5_RGB_LED.pdf): pin 1 common anode, pin 2 blue, 3 green, 4 red cathode. Vf at 20 mA: R 1.8-2.4 V, G/B 2.8-3.6 V. Same 1615 package and pad layout as the common-cathode TJ-S1615SW6TGLCCSRGB-A5 it replaces. LCSC ~13.8k in stock (2026-10-04).</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2129,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>C25744 / C11702 / C25741 exist but showed 0 retail stock at LCSC in one snapshot. Any 0402 1% thick-film resistor of the same value works; JLC Basic stock is separate from LCSC retail. R9/R10 changed 1k -&gt; 100R (0402WGF1000TCE) so green/blue are visible at 3.3 V.</t>
+          <t>C25744 / C11702 / C25741 exist but showed 0 retail stock at LCSC in one snapshot. Any 0402 1% thick-film resistor of the same value works; JLC Basic stock is separate from LCSC retail. R9/R10 changed 1k -&gt; 100R (0402WGF1000TCE) so green/blue are visible at 3.3 V. Draft 3: R9/R10 are 560R (0402WGF5600TCE) in the battery-rail RGB circuit; R15-R17 100k added as FET gate pull-downs.</t>
         </is>
       </c>
     </row>
@@ -2477,7 +2477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2706,6 +2706,23 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>RGB LED: common-cathode from GPIOs (R8 1k, R9/R10 100R) -&gt; common-anode on +BATT with low-side FETs Q3-Q5 (R8 1k, R9/R10 560R, R15-R17 100k pull-downs)</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Green and blue need about 2.6 V at 2 mA (up to 3.0 V worst case) and the 3.3 V rail sags to about 3.0 V on a low battery, so driving them from a 3.3 V GPIO left no headroom whatever the resistor. From the battery (3.0-4.2 V) they stay lit, and no GPIO sees battery voltage. JOT-HW-001 draft 3, section 4.10.</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>D2 -&gt; TJ-S1615SW6TGLCCYRGB-A5 (C273610). Q3/Q4/Q5 AO3400A, gates LED_R/LED_G/LED_B, sources GND, drains via R8/R9/R10 to D2 R/G/B cathodes; D2 anode on +BATT. About 2 mA per colour at 3.7 V. HIGH = on. Changed 2026-10-04.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
NFC sheet: AE1 PCB coil across NFC1/NFC2, C16/C17 180 pF to GND (provisional for ~1.5 uH); title block; BOM row for the NFC caps
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Schematics/RevA/BOM/Jot_RevA_BOM.xlsx
+++ b/Schematics/RevA/BOM/Jot_RevA_BOM.xlsx
@@ -1457,6 +1457,36 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>CL05C181JB5NNNC</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>C16,C17</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>180 pF C0G 0402 (NFC tuning, provisional for a ~1.5 uH coil; recalculate once the coil is drawn)</t>
+        </is>
+      </c>
+    </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
@@ -2298,27 +2328,27 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>C-NFC (x2)</t>
+          <t>C16, C17 (NFC)</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
+          <t>CL05C181JB5NNNC</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C31" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>Not chosen</t>
+          <t>Provisional - 180 pF</t>
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>NFC tuning caps, NFC1/NFC2 to GND, equal values, C0G 0402. Per Nordic nWP-026: Ctune = 2/((2*pi*13.56 MHz)^2 * Lant) - Cp - 4 pF. Starting values: 1.0 uH ~270 pF, 1.5 uH ~180 pF, 2.0 uH ~134 pF. Final value set by tuning the built board (open item 8).</t>
+          <t>NFC tuning caps, NFC1/NFC2 to GND, equal values, C0G 0402. Per Nordic nWP-026: Ctune = 2/((2*pi*13.56 MHz)^2 * Lant) - Cp - 4 pF. Starting values: 1.0 uH ~270 pF, 1.5 uH ~180 pF, 2.0 uH ~134 pF. 180 pF placed on the schematic (2026-10-04) as the 1.5 uH starting value; recalculate from the drawn coil, then final value set by tuning the built board (open item 8).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Schematic review fixes: R18 100k flash /CS pull-up, R19 10R buzzer series resistor, T3902 DATA pin tri-state (ERC clean); BOM quantities and pin list updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Schematics/RevA/BOM/Jot_RevA_BOM.xlsx
+++ b/Schematics/RevA/BOM/Jot_RevA_BOM.xlsx
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1291,7 +1291,7 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
@@ -1310,12 +1310,12 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>R12,R13,R15,R16,R17</t>
+          <t>R12,R13,R15,R16,R17,R18</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>100k 1% 0402 (Q1, Q3, Q4, Q5 gate pull-downs; Q2 gate pull-up)</t>
+          <t>100k 1% 0402 (Q1, Q3, Q4, Q5 gate pull-downs; Q2 gate pull-up; U4 /CS pull-up)</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>C-various</t>
+          <t>C5,C10,C11,C13</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -1381,7 +1381,7 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
@@ -1396,7 +1396,7 @@
       <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>C-various</t>
+          <t>C1,C2,C3,C4,C14,C15</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -1407,7 +1407,7 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
@@ -1422,12 +1422,12 @@
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>C-module</t>
+          <t>C6,C7,C12</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>10 uF 10 V X5R 0603 (U1 VDD/VDDH and VBUS, Raytac ref 8.3)</t>
+          <t>10 uF 10 V X5R 0603 (U1 VDD/VDDH and VBUS, Raytac ref 8.3; U7 accelerometer)</t>
         </is>
       </c>
     </row>
@@ -1488,7 +1488,37 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="A35" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>1206W4F100JT5E</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>UNI-ROYAL</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>R19</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>10R 1% 1206, 0.25 W (buzzer series resistor: limits BZ1 drive at 4.2 V and caps current if Q1 is ever left on)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t>Quantities are per board. LCSC rounds up to each part's minimum order. Blank LCSC numbers: the BOM tool matches on the manufacturer part number.</t>
         </is>
@@ -2139,7 +2169,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>R1-R14</t>
+          <t>R1-R19</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -2159,7 +2189,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>C25744 / C11702 / C25741 exist but showed 0 retail stock at LCSC in one snapshot. Any 0402 1% thick-film resistor of the same value works; JLC Basic stock is separate from LCSC retail. R9/R10 changed 1k -&gt; 100R (0402WGF1000TCE) so green/blue are visible at 3.3 V. Draft 3: R9/R10 are 560R (0402WGF5600TCE) in the battery-rail RGB circuit; R15-R17 100k added as FET gate pull-downs.</t>
+          <t>C25744 / C11702 / C25741 exist but showed 0 retail stock at LCSC in one snapshot. Any 0402 1% thick-film resistor of the same value works; JLC Basic stock is separate from LCSC retail. R9/R10 changed 1k -&gt; 100R (0402WGF1000TCE) so green/blue are visible at 3.3 V. Draft 3: R9/R10 are 560R (0402WGF5600TCE) in the battery-rail RGB circuit; R15-R17 100k added as FET gate pull-downs. Schematic review 2026-10-04: R18 100k /CS pull-up on the flash (Winbond: /CS must track VCC at power-up/down); R19 10R 1206 in series with the buzzer.</t>
         </is>
       </c>
     </row>
@@ -2507,7 +2537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2753,6 +2783,40 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Flash /CS pull-up added: R18 100k QSPI_CSN to +3V3</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Schematic review (Claude + Codex). W25Q01JV: "/CS must track the VCC supply level at power-up and power-down ... a pull-up resistor on /CS can be used". nRF52840 GPIOs float during power-up/reset, so /CS was undefined.</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>R18 100k 0402 on the Storage sheet. No static current while /CS is high. Changed 2026-10-04.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Buzzer series resistor added: R19 10R between +BATT and BZ1 (+)</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Schematic review (Claude + Codex). MLT-5020: rated 3.0 Vo-p, operating 2-4 Vo-p, max 100 mA, coil 12 +/-3 ohm. +BATT reaches 4.2 V, and a stuck-on Q1 would draw about 4.2 / 9 = 0.47 A.</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>R19 10R 1206 (0.25 W). Peak about 4.2 / 22 = 0.19 A. D4 flyback now sits directly across BZ1 (cathode on the BZ1+ side of R19). Firmware must still never hold BUZZER_PWM high. Changed 2026-10-04.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Charger: BQ25101 (0.4 mm BGA, not JLCPCB Economic assemblable) -> MCP73831 SOT-23-5; R6 5.1k PROG (196 mA), R5 removed, C1/C2 4.7 uF; BOM, pin list, architecture draft 4
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Schematics/RevA/BOM/Jot_RevA_BOM.xlsx
+++ b/Schematics/RevA/BOM/Jot_RevA_BOM.xlsx
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -591,17 +591,17 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>BQ25101YFPR</t>
+          <t>MCP73831T-2ACI/OT</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Texas Instruments</t>
+          <t>Microchip</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>C478468</t>
+          <t>C424093</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -611,7 +611,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>1-cell LiPo charger, DSBGA-6</t>
+          <t>1-cell LiPo charger, 4.2 V, tri-state STAT, SOT-23-5</t>
         </is>
       </c>
     </row>
@@ -1097,7 +1097,7 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
@@ -1112,12 +1112,12 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>R1,R2</t>
+          <t>R1,R2,R6</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>5.1k 1% 0402 (USB-C CC)</t>
+          <t>5.1k 1% 0402 (USB-C CC; charger PROG: 1000 V / 5.1k = 196 mA)</t>
         </is>
       </c>
     </row>
@@ -1149,41 +1149,41 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>0402WGF1002TCE</t>
+          <t>CL05A475KP5NRNC</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>UNI-ROYAL</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>C25744</t>
+          <t/>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>C1,C2</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>10k 1% 0402 (charger TS)</t>
+          <t>4.7 uF 10 V X5R 0402 (charger VDD and VBAT; MCP73831 needs at least 4.7 uF on each)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>0402WGF6800TCE</t>
+          <t>0402WGF1001TCE</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -1191,15 +1191,19 @@
           <t>UNI-ROYAL</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>C11702</t>
+        </is>
+      </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>R6</t>
+          <t>R7,R8</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>680R 1% 0402 (charger ISET)</t>
+          <t>1k 1% 0402 (Rec LED, RGB red)</t>
         </is>
       </c>
     </row>
@@ -1209,7 +1213,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>0402WGF1001TCE</t>
+          <t>0402WGF5600TCE</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -1217,29 +1221,25 @@
           <t>UNI-ROYAL</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>C11702</t>
-        </is>
-      </c>
+      <c r="D25" s="2" t="n"/>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>R7,R8</t>
+          <t>R9,R10</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>1k 1% 0402 (Rec LED, RGB red)</t>
+          <t>560R 1% 0402 (RGB green, blue)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>0402WGF5600TCE</t>
+          <t>0402WGF2201TCE</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1247,25 +1247,29 @@
           <t>UNI-ROYAL</t>
         </is>
       </c>
-      <c r="D26" s="2" t="n"/>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>C25879</t>
+        </is>
+      </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>R9,R10</t>
+          <t>R11</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>560R 1% 0402 (RGB green, blue)</t>
+          <t>2.2k 1% 0402 (charge LED)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>0402WGF2201TCE</t>
+          <t>0402WGF1003TCE</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -1275,27 +1279,27 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>C25879</t>
+          <t>C25741</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>R11</t>
+          <t>R12,R13,R15,R16,R17,R18</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2.2k 1% 0402 (charge LED)</t>
+          <t>100k 1% 0402 (Q1, Q3, Q4, Q5 gate pull-downs; Q2 gate pull-up; U4 /CS pull-up)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>0402WGF1003TCE</t>
+          <t>0402WGJ022JTCE</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -1305,47 +1309,47 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>C25741</t>
+          <t>C25158</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>R12,R13,R15,R16,R17,R18</t>
+          <t>R14</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>100k 1% 0402 (Q1, Q3, Q4, Q5 gate pull-downs; Q2 gate pull-up; U4 /CS pull-up)</t>
+          <t>2.2R 5% 0402 (U1 VBUS series, Nordic ref)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>0402WGJ022JTCE</t>
+          <t>CL05B104KO5NNNC</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>UNI-ROYAL</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>C25158</t>
+          <t>C1525</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>R14</t>
+          <t>C5,C10,C11,C13</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2.2R 5% 0402 (U1 VBUS series, Nordic ref)</t>
+          <t>100 nF 16 V X7R 0402 decoupling</t>
         </is>
       </c>
     </row>
@@ -1355,7 +1359,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>CL05B104KO5NNNC</t>
+          <t>CL05A105KA5NQNC</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1363,29 +1367,25 @@
           <t>Samsung</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>C1525</t>
-        </is>
-      </c>
+      <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>C5,C10,C11,C13</t>
+          <t>C3,C4,C14,C15</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>100 nF 16 V X7R 0402 decoupling</t>
+          <t>1 uF 25 V X5R 0402 (U9 LDO in/out; U8 REG and VDD)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>CL05A105KA5NQNC</t>
+          <t>CL10A106KP8NNNC</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -1396,22 +1396,22 @@
       <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>C1,C2,C3,C4,C14,C15</t>
+          <t>C6,C7,C12</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>1 uF 25 V X5R 0402 (includes U9 LDO in/out)</t>
+          <t>10 uF 10 V X5R 0603 (U1 VDD/VDDH and VBUS, Raytac ref 8.3; U7 accelerometer)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>CL10A106KP8NNNC</t>
+          <t>CL05C180JB5NNNC</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1422,12 +1422,12 @@
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>C6,C7,C12</t>
+          <t>C-xtal</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>10 uF 10 V X5R 0603 (U1 VDD/VDDH and VBUS, Raytac ref 8.3; U7 accelerometer)</t>
+          <t>18 pF C0G 0402 (32.768 kHz load caps; checked against nRF52840 PS)</t>
         </is>
       </c>
     </row>
@@ -1437,7 +1437,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>CL05C180JB5NNNC</t>
+          <t>CL05C181JB5NNNC</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -1445,30 +1445,34 @@
           <t>Samsung</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr"/>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>C-xtal</t>
+          <t>C16,C17</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>18 pF C0G 0402 (32.768 kHz load caps; checked against nRF52840 PS)</t>
+          <t>180 pF C0G 0402 (NFC tuning, provisional for a ~1.5 uH coil; recalculate once the coil is drawn)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>CL05C181JB5NNNC</t>
+          <t>1206W4F100JT5E</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>UNI-ROYAL</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1478,47 +1482,17 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>C16,C17</t>
+          <t>R19</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>180 pF C0G 0402 (NFC tuning, provisional for a ~1.5 uH coil; recalculate once the coil is drawn)</t>
+          <t>10R 1% 1206, 0.25 W (buzzer series resistor: limits BZ1 drive at 4.2 V and caps current if Q1 is ever left on)</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>1206W4F100JT5E</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>UNI-ROYAL</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>R19</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>10R 1% 1206, 0.25 W (buzzer series resistor: limits BZ1 drive at 4.2 V and caps current if Q1 is ever left on)</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="3" t="inlineStr">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>Quantities are per board. LCSC rounds up to each part's minimum order. Blank LCSC numbers: the BOM tool matches on the manufacturer part number.</t>
         </is>
@@ -1661,22 +1635,22 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>BQ25101YFPR</t>
+          <t>MCP73831T-2ACI/OT</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>C478468</t>
+          <t>C424093</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Verified</t>
+          <t>Verified - datasheet read</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>LCSC datasheet C478468 read: 4.2 V, CHG pin, 10-250 mA. ISET: KISET 135 / 680R = ~200 mA (0.5C for 400 mAh). TS: 10k to VSS is TI's no-thermistor connection.</t>
+          <t>Replaces BQ25101YFPR (2026-10-05): its DSBGA-6 has 0.4 mm ball pitch, below JLCPCB Economic PCBA minimum BGA pitch of 0.5 mm, and cannot be hand-reworked. MCP73831 datasheet (Datasheets/Power/MCP73831_Microchip.pdf): SOT-23-5 pins 1 STAT, 2 VSS, 3 VBAT, 4 VDD, 5 PROG; IREG = 1000 V / RPROG -&gt; 5.1k = 196 mA (0.5C for 400 mAh); STAT low = charging, high = complete (drives D3 from VBUS via R11); min 4.7 uF on VDD and VBAT; battery discharge current 0.15 uA typ / 2 uA max with VDD floating. No TS input (pack has no NTC). LCSC: ~8.9k in stock.</t>
         </is>
       </c>
     </row>
@@ -2537,7 +2511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2817,6 +2791,23 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Charger: TI BQ25101YFPR (DSBGA-6) -&gt; Microchip MCP73831T-2ACI/OT (SOT-23-5)</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Caught before footprints: the BQ25101 DSBGA has 0.4 mm ball pitch. JLCPCB Economic PCBA only places BGAs down to 0.5 mm; Standard PCBA can, but needs a 70 x 70 mm minimum piece (a panel of ~8-12 Jots) at higher cost. A 0.4 mm BGA also cannot be reworked by hand on a first board.</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>U5 MCP73831 (KiCad Battery_Management:MCP73831-2-OT). R6 680R -&gt; 5.1k PROG (196 mA). R5 (TS) removed. C1/C2 1 uF -&gt; 4.7 uF. Charge LED unchanged on STAT. Loses battery-temperature input (pack has no NTC anyway). Changed 2026-10-05.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
BOM: LCSC numbers on every line; stock note updated from the 2026-10-05 assembly check
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Schematics/RevA/BOM/Jot_RevA_BOM.xlsx
+++ b/Schematics/RevA/BOM/Jot_RevA_BOM.xlsx
@@ -1109,7 +1109,11 @@
           <t>UNI-ROYAL</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr"/>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>C25905</t>
+        </is>
+      </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
           <t>R1,R2,R6</t>
@@ -1135,7 +1139,11 @@
           <t>UNI-ROYAL</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>C25900</t>
+        </is>
+      </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
           <t>R3,R4</t>
@@ -1163,7 +1171,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>C368809</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1221,7 +1229,11 @@
           <t>UNI-ROYAL</t>
         </is>
       </c>
-      <c r="D25" s="2" t="n"/>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>C25126</t>
+        </is>
+      </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
           <t>R9,R10</t>
@@ -1367,7 +1379,11 @@
           <t>Samsung</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>C52923</t>
+        </is>
+      </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
           <t>C3,C4,C14,C15</t>
@@ -1393,7 +1409,11 @@
           <t>Samsung</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr"/>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>C19702</t>
+        </is>
+      </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
           <t>C6,C7,C12</t>
@@ -1419,7 +1439,11 @@
           <t>Samsung</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>C307443</t>
+        </is>
+      </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
           <t>C8,C9</t>
@@ -1447,7 +1471,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>C12209</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1477,7 +1501,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>C17903</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -2158,12 +2182,12 @@
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Verified exists - stock fluctuates</t>
+          <t>Verified - in stock (JLCPCB parts library, 2026-10-05)</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>C25744 / C11702 / C25741 exist but showed 0 retail stock at LCSC in one snapshot. Any 0402 1% thick-film resistor of the same value works; JLC Basic stock is separate from LCSC retail. R9/R10 changed 1k -&gt; 100R (0402WGF1000TCE) so green/blue are visible at 3.3 V. Draft 3: R9/R10 are 560R (0402WGF5600TCE) in the battery-rail RGB circuit; R15-R17 100k added as FET gate pull-downs. Schematic review 2026-10-04: R18 100k /CS pull-up on the flash (Winbond: /CS must track VCC at power-up/down); R19 10R 1206 in series with the buzzer.</t>
+          <t>All in stock in the JLCPCB parts library (2026-10-05 assembly check). Any 0402 1% thick-film resistor of the same value works; JLC Basic stock is separate from LCSC retail. R9/R10 changed 1k -&gt; 100R (0402WGF1000TCE) so green/blue are visible at 3.3 V. Draft 3: R9/R10 are 560R (0402WGF5600TCE) in the battery-rail RGB circuit; R15-R17 100k added as FET gate pull-downs. Schematic review 2026-10-04: R18 100k /CS pull-up on the flash (Winbond: /CS must track VCC at power-up/down); R19 10R 1206 in series with the buzzer.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rev A schematic final: battery fuse, reverse protection, VBUS TVS, charge inhibit, 32 MB flash
Polyfuse F1 and reverse-polarity P-FET Q6 between J2 and +BATT; SMF5.0A TVS on
VBUS; firmware charge inhibit (Q7/Q8, R20/R21, CHG_INHIBIT on P1.11, charging on
by default); R19 10R 1 W 2512; I2C pull-ups 2.2k; 1k series resistor on BTN;
flash W25Q256JVEIQ (symbol renamed); TP1/TP2/TP6 and J2 labels; junction dots.
BOM, pin list and architecture draft 5 updated (section 4.14: protection summary
and known Rev A limitations). JLCPCB upload BOM added. ERC clean.
</commit_message>
<xml_diff>
--- a/Schematics/RevA/BOM/Jot_RevA_BOM.xlsx
+++ b/Schematics/RevA/BOM/Jot_RevA_BOM.xlsx
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -561,7 +561,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>W25Q01JVZEIQ</t>
+          <t>W25Q256JVEIQ</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -571,7 +571,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>C5137036</t>
+          <t>C97522</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -581,7 +581,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>1 Gbit (128 MB) QSPI NOR flash, WSON-8 8x6 mm</t>
+          <t>256 Mbit (32 MB) QSPI NOR flash, WSON-8 8x6 mm (about 68 min of 8 KB/s audio)</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Haptic driver, VSSOP-10</t>
+          <t>Haptic driver, VSSOP-10 (pre-ordered at JLCPCB 8 Oct: low stock)</t>
         </is>
       </c>
     </row>
@@ -767,7 +767,7 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
@@ -786,18 +786,18 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q2,Q6</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>P-MOSFET, mic + Rec LED power switch, SOT-23</t>
+          <t>P-MOSFET, SOT-23: mic + Rec LED power switch (Q2); battery reverse-polarity protection (Q6, gate to GND)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
@@ -816,12 +816,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Q1,Q3,Q4,Q5</t>
+          <t>Q1,Q3,Q4,Q5,Q7,Q8</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>N-MOSFET, SOT-23: buzzer driver (Q1) and RGB LED cathode switches (Q3-Q5)</t>
+          <t>N-MOSFET, SOT-23: buzzer driver (Q1), RGB cathode switches (Q3-Q5), charge inhibit (Q7 in the PROG path, Q8 driven by CHG_INHIBIT)</t>
         </is>
       </c>
     </row>
@@ -1131,57 +1131,57 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>0402WGF4701TCE</t>
+          <t>CL05A475KP5NRNC</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>UNI-ROYAL</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>C25900</t>
+          <t>C368809</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>R3,R4</t>
+          <t>C1,C2</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>4.7k 1% 0402 (I2C pull-ups)</t>
+          <t>4.7 uF 10 V X5R 0402 (charger VDD and VBAT; MCP73831 needs at least 4.7 uF on each)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>CL05A475KP5NRNC</t>
+          <t>0402WGF1001TCE</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>UNI-ROYAL</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>C368809</t>
+          <t>C11702</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>C1,C2</t>
+          <t>R5,R7,R8</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>4.7 uF 10 V X5R 0402 (charger VDD and VBAT; MCP73831 needs at least 4.7 uF on each)</t>
+          <t>1k 1% 0402 (R5 BTN series ESD resistor; Rec LED; RGB red)</t>
         </is>
       </c>
     </row>
@@ -1191,7 +1191,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>0402WGF1001TCE</t>
+          <t>0402WGF5600TCE</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -1201,27 +1201,27 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>C11702</t>
+          <t>C25126</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>R7,R8</t>
+          <t>R9,R10</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>1k 1% 0402 (Rec LED, RGB red)</t>
+          <t>560R 1% 0402 (RGB green, blue)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>0402WGF5600TCE</t>
+          <t>0402WGF2201TCE</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -1231,27 +1231,27 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>C25126</t>
+          <t>C25879</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>R9,R10</t>
+          <t>R3,R4,R11</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>560R 1% 0402 (RGB green, blue)</t>
+          <t>2.2k 1% 0402 (I2C pull-ups R3/R4: MAX17048 60 pF + 300 ns rise; charge LED R11)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>0402WGF2201TCE</t>
+          <t>0402WGF1003TCE</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1261,27 +1261,27 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>C25879</t>
+          <t>C25741</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>R11</t>
+          <t>R12,R13,R15,R16,R17,R18,R20,R21</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2.2k 1% 0402 (charge LED)</t>
+          <t>100k 1% 0402 (Q1, Q3-Q5 gate pull-downs; Q2 gate pull-up; U4 /CS pull-up; R20 Q7 gate to VBUS; R21 CHG_INHIBIT pull-down)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>0402WGF1003TCE</t>
+          <t>0402WGJ022JTCE</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -1291,47 +1291,47 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>C25741</t>
+          <t>C25158</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>R12,R13,R15,R16,R17,R18</t>
+          <t>R14</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>100k 1% 0402 (Q1, Q3, Q4, Q5 gate pull-downs; Q2 gate pull-up; U4 /CS pull-up)</t>
+          <t>2.2R 5% 0402 (U1 VBUS series, Nordic ref)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>0402WGJ022JTCE</t>
+          <t>CL05B104KO5NNNC</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>UNI-ROYAL</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>C25158</t>
+          <t>C1525</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>R14</t>
+          <t>C5,C10,C11,C13</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2.2R 5% 0402 (U1 VBUS series, Nordic ref)</t>
+          <t>100 nF 16 V X7R 0402 decoupling</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>CL05B104KO5NNNC</t>
+          <t>CL05A105KA5NQNC</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -1351,27 +1351,27 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>C1525</t>
+          <t>C52923</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>C5,C10,C11,C13</t>
+          <t>C3,C4,C14,C15</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>100 nF 16 V X7R 0402 decoupling</t>
+          <t>1 uF 25 V X5R 0402 (U9 LDO in/out; U8 REG and VDD)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>CL05A105KA5NQNC</t>
+          <t>CL10A106KP8NNNC</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1381,27 +1381,27 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>C52923</t>
+          <t>C19702</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>C3,C4,C14,C15</t>
+          <t>C6,C7,C12</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>1 uF 25 V X5R 0402 (U9 LDO in/out; U8 REG and VDD)</t>
+          <t>10 uF 10 V X5R 0603 (U1 VDD/VDDH and VBUS, Raytac ref 8.3; U7 accelerometer)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>CL10A106KP8NNNC</t>
+          <t>CL05C180JB5NNNC</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -1411,17 +1411,17 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>C19702</t>
+          <t>C307443</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>C6,C7,C12</t>
+          <t>C8,C9</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>10 uF 10 V X5R 0603 (U1 VDD/VDDH and VBUS, Raytac ref 8.3; U7 accelerometer)</t>
+          <t>18 pF C0G 0402 (32.768 kHz load caps; checked against nRF52840 PS)</t>
         </is>
       </c>
     </row>
@@ -1431,7 +1431,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>CL05C180JB5NNNC</t>
+          <t>CL05C181JB5NNNC</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1441,82 +1441,142 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>C307443</t>
+          <t>C12209</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>C8,C9</t>
+          <t>C16,C17</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>18 pF C0G 0402 (32.768 kHz load caps; checked against nRF52840 PS)</t>
+          <t>180 pF C0G 0402 (NFC tuning, provisional for a ~1.5 uH coil; recalculate once the coil is drawn)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>CL05C181JB5NNNC</t>
+          <t>25121WF100JT4E</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>UNI-ROYAL</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>C12209</t>
+          <t>C47019</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>C16,C17</t>
+          <t>R19</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>180 pF C0G 0402 (NFC tuning, provisional for a ~1.5 uH coil; recalculate once the coil is drawn)</t>
+          <t>10R 1% 2512, 1 W (buzzer series resistor; survives a stuck-on Q1: 0.49 W)</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n">
+      <c r="A34" t="n">
         <v>1</v>
       </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>1206W4F100JT5E</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>UNI-ROYAL</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>C17903</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>R19</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>10R 1% 1206, 0.25 W (buzzer series resistor: limits BZ1 drive at 4.2 V and caps current if Q1 is ever left on)</t>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>MDBT50Q-1MV2</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Raytac</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>C5118826</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>U1</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>nRF52840 module, chip antenna (pre-ordered at JLCPCB 8 Oct, held in My Parts)</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="A35" t="n">
+        <v>1</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>SMD0805P050TF</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>RUILON</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>C20978</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Polyfuse 0.5 A hold / 1 A trip, 6 V, 0805 (battery rail; 0.33 A hold at 60 C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>1</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>SMF5.0A</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>MDD</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>C193402</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>TVS 5 V standoff, 6.4-7 V breakdown, unidirectional, SOD-123FL (VBUS hot-plug; cathode to VBUS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>Quantities are per board. LCSC rounds up to each part's minimum order. Blank LCSC numbers: the BOM tool matches on the manufacturer part number.</t>
         </is>
@@ -1533,7 +1593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1632,22 +1692,22 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>W25Q01JVZEIQ</t>
+          <t>W25Q256JVEIQ</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>C5137036</t>
+          <t>C97522</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Verified</t>
+          <t>Verified - datasheet read</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>LCSC datasheet C5137036 read: 1 Gbit, 2.7-3.6 V, IQ = quad enabled. Two stacked 512 Mbit dies with linear 4-byte addressing; BUSY is reported per die. Program/erase up to 25 mA.</t>
+          <t>Replaces W25Q01JVZEIQ (C5137036, $36.51, 231 in stock) on 8 Oct: $4.34, ~2.5k in stock. Same WSON-8 8x6 package and pinout (Datasheets/Storage/W25Q256JV_Winbond.pdf): pin 7 /HOLD-/RESET/IO3; QE = 1 fixed for IQ. 2.7-3.6 V. Powers up in 3-byte addressing: firmware enters 4-byte mode (B7h). Read voltage must stay within +/-10% of the program voltage: no writes below the low-battery cutoff.</t>
         </is>
       </c>
     </row>
@@ -1755,7 +1815,7 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>LCSC page: ~4,500 in stock.</t>
+          <t>Only 58 in JLCPCB stock on 8 Oct: 7 pre-ordered (C527464).</t>
         </is>
       </c>
     </row>
@@ -1843,7 +1903,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Q1, Q3-Q5</t>
+          <t>Q1, Q3-Q5, Q7, Q8</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -1863,14 +1923,14 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Replaces 2N7002: buzzer can draw ~100 mA and 2N7002 is only rated 115 mA with 2.5 V threshold. AO3400A is logic-level. Draft 3: the same part switches the RGB LED cathodes (Q3-Q5), gate from a 3.3 V GPIO with a 100k pull-down.</t>
+          <t>Replaces 2N7002: buzzer can draw ~100 mA and 2N7002 is only rated 115 mA with 2.5 V threshold. AO3400A is logic-level. Draft 3: the same part switches the RGB LED cathodes (Q3-Q5), gate from a 3.3 V GPIO with a 100k pull-down. Q7/Q8 (8 Oct): charge inhibit.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q2, Q6</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -1890,7 +1950,7 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>UMW version chosen: &gt;500k stock. (AOS C15127 is marked NRND on LCSC.) Gate low = on.</t>
+          <t>UMW version chosen: &gt;500k stock. (AOS C15127 is marked NRND on LCSC.) Gate low = on. Q6 (8 Oct): reverse-battery P-FET, D to BATT_FUSED, S to +BATT, G to GND. Vds -30 V, Vgs +/-12 V, Rds(on) &lt; 120 mOhm at -2.5 V.</t>
         </is>
       </c>
     </row>
@@ -2290,12 +2350,12 @@
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>Not from LCSC</t>
+          <t>Pre-ordered</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>Out of stock at LCSC. Buy from DigiKey/Mouser; hand-solder or consign to JLC. Raytac datasheet Ver L read: every module pin number in the pin list matches; ref circuit 8.3 (external 3.3 V) used for decoupling.</t>
+          <t>Pre-ordered at JLCPCB 8 Oct (6 pcs, ~$18.25, ~15-day lead) so it sits in My Parts for the PCBA order. TME had 702 at $9.45 as a fallback. Raytac datasheet Ver L read: every module pin matches; ref circuit 8.3; antenna keep-out section 2.3.</t>
         </is>
       </c>
     </row>
@@ -2377,6 +2437,141 @@
       <c r="E31" s="6" t="inlineStr">
         <is>
           <t>NFC tuning caps, NFC1/NFC2 to GND, equal values, C0G 0402. Per Nordic nWP-026: Ctune = 2/((2*pi*13.56 MHz)^2 * Lant) - Cp - 4 pF. Starting values: 1.0 uH ~270 pF, 1.5 uH ~180 pF, 2.0 uH ~134 pF. 180 pF placed on the schematic (2026-10-04) as the 1.5 uH starting value; recalculate from the drawn coil, then final value set by tuning the built board (open item 8).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>SMD0805P050TF</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>C20978</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Verified - datasheet read</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Added 8 Oct (senior review). Datasheets/Power/SMD0805P050TF_Polyfuse.pdf: hold 0.50 A / trip 1.0 A at 25 C; hold 0.40 A at 40 C, 0.33 A at 60 C, 0.23 A at 85 C; 6 V. Worst sustained load ~245 mA, charging ~200 mA. Trips below the pack protection (2-5 A).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>SMF5.0A</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>C193402</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Verified - datasheet read</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Added 8 Oct. MCP73831 6.1.1.2: input overvoltage protection must be used for hot-plugged USB. Standoff 5 V, breakdown 6.4-7 V, clamp 9.2 V at 21.7 A (Littelfuse SMF datasheet in Datasheets/Power; MDD C193402 has the same ratings). Does not guarantee &lt;5.8 V at the nRF VBUS pin in a large surge: Rev A known limitation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>R19</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>25121WF100JT4E</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>C47019</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>8 Oct: 1206 0.25 W -&gt; 2512 1 W. Stuck-on Q1: 0.22 A, 0.49 W. A short at BZ1+ to GND (1.76 W) still exceeds it: manufacturing fault, inspect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>R20, R21, Q7, Q8</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>100k / AO3400A</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>C25741 / C20917</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>8 Oct charge inhibit: PROG -&gt; R6 -&gt; Q7 -&gt; GND; R20 pulls Q7 gate to VBUS (charging by default, even with the MCU unpowered); Q8 (gate CHG_INHIBIT = U1 P1.11, R21 pull-down) pulls Q7 gate low to float PROG and stop charging (MCP73831 3.5 / 4.3).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>0402WGF1001TCE</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>C11702</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>8 Oct: 1k in series with BTN (ESD). Reuses the R5 designator retired with the BQ25101 on 5 Oct. Pressed level ~0.24 V with the ~13k internal pull-up.</t>
         </is>
       </c>
     </row>
@@ -2391,7 +2586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2437,12 +2632,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Raytac MDBT50Q-1MV2</t>
+          <t>Vybronics VG0832012</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
@@ -2450,29 +2645,29 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>DigiKey / Mouser</t>
+          <t>DigiKey</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>MDBT50Q-1MV2</t>
+          <t>1670-VG0832012-ND</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>nRF52840 module, chip antenna</t>
+          <t>LRA, wire leads, hand-solder</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>BT1</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Vybronics VG0832012</t>
+          <t>Adafruit 3898</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
@@ -2485,40 +2680,10 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>1670-VG0832012-ND</t>
+          <t>1528-2731-ND</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>LRA, wire leads, hand-solder</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>BT1</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Adafruit 3898</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>DigiKey</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>1528-2731-ND</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>400 mAh LiPo, JST-PH, ground ship only</t>
         </is>
@@ -2535,7 +2700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2832,6 +2997,125 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Polyfuse F1 + reverse-polarity Q6 between J2 and +BATT (8 Oct)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Coworker review (Ben) and Claude + Codex senior review: the battery rail had no protection below the pack trip (2-5 A), and no reverse-battery protection.</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>J2 pin 1 -&gt; BATT_RAW -&gt; F1 SMD0805P050TF -&gt; BATT_FUSED -&gt; Q6 AO3401A (D) -&gt; (S) +BATT, Q6 gate GND. Limitation: with USB present a reversed pack can still take ~20 mA (Rev B: ideal-diode switch).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>TVS D5 on VBUS (8 Oct)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>MCP73831 6.1.1.2 requires input overvoltage protection for hot-plug USB.</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>D5 SMF5.0A, cathode VBUS, anode GND, next to J1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Charge inhibit Q7/Q8, R20/R21 (8 Oct)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Battery may only charge at 0-45 C; MCP73831 has no temperature input. Firmware stops charging from the nRF/accelerometer temperature.</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>CHG_INHIBIT (U1 P1.11) high = charging off. Default (MCU off/reset) = charging on. Limitation: not cell temperature and inactive while the MCU is off (Rev B: NTC charger).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>R19 1206 0.25 W -&gt; 2512 1 W (8 Oct)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Stuck-on Q1 puts 0.49 W in R19.</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Footprint R_2512_6332Metric. Firmware: buzzer only via PWM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>I2C pull-ups R3/R4 4.7k -&gt; 2.2k (8 Oct)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>MAX17048: up to 60 pF input capacitance and 300 ns max rise time left ~15 pF margin at 4.7k (Ben, Codex).</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Same part as R11 (C25879).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>BTN series resistor R5 1k (8 Oct)</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ESD on the one part people press; units will be given to people.</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>U1 P1.10 -&gt; BTN -&gt; R5 -&gt; SW1 -&gt; GND.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Flash W25Q01JVZEIQ -&gt; W25Q256JVEIQ (8 Oct)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>$36.51 -&gt; $4.34 per board; 32 MB is ~68 min of audio, enough between syncs.</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Same footprint and pinout. Firmware: 4-byte addressing.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Architecture and BOM: neutral review wording
</commit_message>
<xml_diff>
--- a/Schematics/RevA/BOM/Jot_RevA_BOM.xlsx
+++ b/Schematics/RevA/BOM/Jot_RevA_BOM.xlsx
@@ -2954,7 +2954,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Schematic review (Claude + Codex). W25Q01JV: "/CS must track the VCC supply level at power-up and power-down ... a pull-up resistor on /CS can be used". nRF52840 GPIOs float during power-up/reset, so /CS was undefined.</t>
+          <t>Schematic review. W25Q01JV: "/CS must track the VCC supply level at power-up and power-down ... a pull-up resistor on /CS can be used". nRF52840 GPIOs float during power-up/reset, so /CS was undefined.</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2971,7 +2971,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Schematic review (Claude + Codex). MLT-5020: rated 3.0 Vo-p, operating 2-4 Vo-p, max 100 mA, coil 12 +/-3 ohm. +BATT reaches 4.2 V, and a stuck-on Q1 would draw about 4.2 / 9 = 0.47 A.</t>
+          <t>Schematic review. MLT-5020: rated 3.0 Vo-p, operating 2-4 Vo-p, max 100 mA, coil 12 +/-3 ohm. +BATT reaches 4.2 V, and a stuck-on Q1 would draw about 4.2 / 9 = 0.47 A.</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -3005,7 +3005,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Coworker review (Ben) and Claude + Codex senior review: the battery rail had no protection below the pack trip (2-5 A), and no reverse-battery protection.</t>
+          <t>Fault-by-fault design review: the battery rail had no protection below the pack trip (2-5 A), and no reverse-battery protection.</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -3073,7 +3073,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>MAX17048: up to 60 pF input capacitance and 300 ns max rise time left ~15 pF margin at 4.7k (Ben, Codex).</t>
+          <t>MAX17048: up to 60 pF input capacitance and 300 ns max rise time left ~15 pF margin at 4.7k.</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">

</xml_diff>

<commit_message>
Battery: Adafruit 1578 (PKCELL LP503035, 500 mAh, 30 x 35 x 5.0 mm) replaces the 3898
Datasheet filed; BOM (Buy Elsewhere, Verification, Design Changes), architecture
draft 5 and the case battery pocket updated. Pocket sized to the drawing maximum
and moved 1.5 mm up to clear the bottom screw posts.
</commit_message>
<xml_diff>
--- a/Schematics/RevA/BOM/Jot_RevA_BOM.xlsx
+++ b/Schematics/RevA/BOM/Jot_RevA_BOM.xlsx
@@ -1734,7 +1734,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Replaces BQ25101YFPR (2026-10-05): its DSBGA-6 has 0.4 mm ball pitch, below JLCPCB Economic PCBA minimum BGA pitch of 0.5 mm, and cannot be hand-reworked. MCP73831 datasheet (Datasheets/Power/MCP73831_Microchip.pdf): SOT-23-5 pins 1 STAT, 2 VSS, 3 VBAT, 4 VDD, 5 PROG; IREG = 1000 V / RPROG -&gt; 5.1k = 196 mA (0.5C for 400 mAh); STAT low = charging, high = complete (drives D3 from VBUS via R11); min 4.7 uF on VDD and VBAT; battery discharge current 0.15 uA typ / 2 uA max with VDD floating. No TS input (pack has no NTC). LCSC: ~8.9k in stock.</t>
+          <t>Replaces BQ25101YFPR (2026-10-05): its DSBGA-6 has 0.4 mm ball pitch, below JLCPCB Economic PCBA minimum BGA pitch of 0.5 mm, and cannot be hand-reworked. MCP73831 datasheet (Datasheets/Power/MCP73831_Microchip.pdf): SOT-23-5 pins 1 STAT, 2 VSS, 3 VBAT, 4 VDD, 5 PROG; IREG = 1000 V / RPROG -&gt; 5.1k = 196 mA (0.39C for the 500 mAh Adafruit 1578; 0.5C for the original 400 mAh pack); STAT low = charging, high = complete (drives D3 from VBUS via R11); min 4.7 uF on VDD and VBAT; battery discharge current 0.15 uA typ / 2 uA max with VDD floating. No TS input (pack has no NTC). LCSC: ~8.9k in stock.</t>
         </is>
       </c>
     </row>
@@ -2394,7 +2394,7 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Adafruit 3898</t>
+          <t>Adafruit 1578 (PKCELL LP503035)</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
@@ -2404,12 +2404,12 @@
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>Not from LCSC</t>
+          <t>Verified - datasheet read</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>DigiKey 1528-2731-ND.</t>
+          <t>Replaces Adafruit 3898 (36 x 17 x 7.8 mm, 400 mAh) on 8 Oct so the case is 12.8 mm thick, not 16. Datasheets/Power/Adafruit_1578_LP503035_500mAh.pdf (PKCELL QA.S.0228): 500 mAh (450 min), 4.2 V charge, standard 0.2C, quick 1C (500 mA) -&gt; MCP73831 196 mA = 0.39C OK; max continuous discharge 1C (500 mA) vs ~245 mA worst sustained; charge 0-45 C (charge inhibit in firmware); PCM S-8261AAJMD + MOSFET 8814; drawing 30 +/-0.1 x 35 +/-0.1 x 5.0 +/-0.1 mm incl. PCM (Adafruit page says 29 x 36 x 4.75; case designed to the drawing max); JST PH-2P "reverse the plug" = Adafruit polarity, matching J2 pin 1 = +; leads 100 mm red/black 24 AWG from a 30 mm end. In stock at Adafruit 8 Oct, $7.95.</t>
         </is>
       </c>
     </row>
@@ -2667,7 +2667,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Adafruit 3898</t>
+          <t>Adafruit 1578 (PKCELL LP503035)</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
@@ -2675,17 +2675,17 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>DigiKey</t>
+          <t>Adafruit (adafruit.com/product/1578, $7.95)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>1528-2731-ND</t>
+          <t>1578</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>400 mAh LiPo, JST-PH, ground ship only</t>
+          <t>500 mAh LiPo, 30 x 35 x 5.0 mm (+/-0.1), protection board (S-8261), JST-PH 2-pin with Adafruit polarity (pin 1 = +), 100 mm leads. Ground ship only. Check polarity with a meter before first plug-in.</t>
         </is>
       </c>
     </row>
@@ -2700,7 +2700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3116,6 +3116,23 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Battery: Adafruit 3898 (400 mAh, 7.8 mm thick) -&gt; Adafruit 1578 (500 mAh, 5.0 mm thick) (8 Oct)</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Case thickness: the 7.8 mm cell made the case 16 mm thick; the 5.0 mm cell brings it to 12.8 mm with more capacity. Same maker, same JST-PH polarity.</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>No schematic change (J2 unchanged). Case battery pocket 30.1 x 35.1 mm, moved 1.5 mm up to clear the bottom screw posts. Put J2 near the battery lead end at layout.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rev A layout: net classes, ground plane and vias, main 5 V path; NFC paperwork
- Net classes: Default 0.2 mm / 0.15 mm clearance; Power 0.5 mm for VBUS,
  +BATT, BATT_RAW, BATT_FUSED and the buzzer nets
- In1.Cu solid GND zone (antenna keep-out respected); U7 pad clearance
  override removed
- 43 GND vias, every GND pad tied to the plane on F.Cu, no via-in-pad
- VBUS: J1 -> D5 -> C1 and across to the charger U5, 0.5 mm on F.Cu, kept
  clear of the USB CC and data pins; J1's second VBUS pin and U10 pin 5 to
  follow on B.Cu
- BOM and JLCPCB BOM: C16/C17 82 pF YAGEO CC0402JRNPO9BN820 (C107011),
  C18/C19 DNP tuning pads, AE1 Molex 146236-0101 bought separately
- Architecture draft 6: NFC section rewritten for the flex antenna
</commit_message>
<xml_diff>
--- a/Schematics/RevA/BOM/Jot_RevA_BOM.xlsx
+++ b/Schematics/RevA/BOM/Jot_RevA_BOM.xlsx
@@ -1431,17 +1431,17 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>CL05C181JB5NNNC</t>
+          <t>CC0402JRNPO9BN820</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>C12209</t>
+          <t>C107011</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1451,7 +1451,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>180 pF C0G 0402 (NFC tuning, provisional for a ~1.5 uH coil; recalculate once the coil is drawn)</t>
+          <t>82 pF 5% NP0 50 V 0402 (NFC tuning for the Molex 146236-0101 antenna, 3.1 uH; Nordic nRF52840 PS p.461). Extended part: no Basic 82 pF 0402 exists.</t>
         </is>
       </c>
     </row>
@@ -1593,7 +1593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2421,22 +2421,22 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>CL05C181JB5NNNC</t>
+          <t>CC0402JRNPO9BN820</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>C107011</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>Provisional - 180 pF</t>
+          <t>Verified - calculated</t>
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>NFC tuning caps, NFC1/NFC2 to GND, equal values, C0G 0402. Per Nordic nWP-026: Ctune = 2/((2*pi*13.56 MHz)^2 * Lant) - Cp - 4 pF. Starting values: 1.0 uH ~270 pF, 1.5 uH ~180 pF, 2.0 uH ~134 pF. 180 pF placed on the schematic (2026-10-04) as the 1.5 uH starting value; recalculate from the drawn coil, then final value set by tuning the built board (open item 8).</t>
+          <t>14 Oct: 180 pF -&gt; 82 pF for the Molex 146236-0101 flex antenna (L = 3.1 uH, Molex PS-1462360001). Nordic nRF52840 PS v1.11 6.14.10 p.461: Ctune = 2/((2*pi*13.56 MHz)^2 * L) - Cp - Cint = 88.9 - 2 - 4 = 82.9 pF. The battery behind the ferrite will shift L, so tune on the first board with C18/C19. JLCPCB parts API 14 Oct: Extended, 260k in stock.</t>
         </is>
       </c>
     </row>
@@ -2572,6 +2572,60 @@
       <c r="E36" t="inlineStr">
         <is>
           <t>8 Oct: 1k in series with BTN (ESD). Reuses the R5 designator retired with the BQ25101 on 5 Oct. Pressed level ~0.24 V with the ~13k internal pull-up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>C18, C19 (NFC)</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>DNP</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Spare 0402 pads in parallel with C16/C17 for hand-tuning the NFC antenna on the built board. Not assembled; excluded from BOM and placement file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>AE1 (NFC)</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Molex 146236-0101</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Not from LCSC</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Flex NFC antenna with ferrite, 15 x 25 mm + solder-pad tab, 0.27 mm, 3.1 uH, Q 51.8. Stuck in the back-shell pocket, wires through the AE1 holes (SolderWire 0.1 sqmm). DigiKey/Newark stock seen 8 Oct; confirm before ordering.</t>
         </is>
       </c>
     </row>
@@ -2586,7 +2640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2689,6 +2743,38 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>AE1</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Molex 146236-0101</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>DigiKey or Newark</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>146236-0101</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>NFC flex antenna with ferrite, 15 x 25 mm + tab, 0.27 mm thick, 3.1 uH. Two fine wires from its pads to the AE1 holes. Solder quickly (thin polyimide tab).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2700,7 +2786,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3133,6 +3219,23 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>NFC antenna: PCB coil -&gt; Molex 146236-0101 flex antenna (8 Oct)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>A PCB coil needs ~20 x 20 mm with no copper on any layer, and the only metal-free area is the BLE antenna corner. A ferrite-backed flex antenna in the back shell takes no board space and works over the battery.</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>AE1 -&gt; 2 solder-wire holes at the right edge (12 mm from the BLE antenna). C16/C17 180 pF -&gt; 82 pF. C18/C19 added as DNP tuning pads. Tap the back of Jot on the phone.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rev A layout complete: final routing and layout review fixes
- J2 is now two solder-wire holes (battery leads soldered): the JST-PH
  side-entry header is 5.5 mm tall and would not fit the 12.8 mm case.
  Removed from the JLCPCB BOM; BOM, architecture doc and case notes updated.
- LED drive pins re-assigned to match the transistor order:
  P1.08 red, P0.11 green, P0.12 blue. Pin list updated.
- No via drilled inside an SMD pad; no top-layer signal or via beside the
  crystal; 5 V branch removed from the power layer under the USB pair.
- R19 off the battery, C11 next to the mic, short ground vias at the
  module and decoupling capacitors, clean reset route.
- Silkscreen labels at 1.0 mm, battery + / - marked; zones refilled.
- DRC clean, board matches schematic, ERC clean.
- Case: 0.4 mm pocket over SW1, lip 0.8 mm.
- Architecture draft 7.
</commit_message>
<xml_diff>
--- a/Schematics/RevA/BOM/Jot_RevA_BOM.xlsx
+++ b/Schematics/RevA/BOM/Jot_RevA_BOM.xlsx
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -891,27 +891,27 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>S2B-PH-SM4-TB(LF)(SN)</t>
+          <t>TS-1010-C-A</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>C295747</t>
+          <t>C692458</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>J2</t>
+          <t>SW1</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>JST-PH 2-pin battery connector, SMD right angle</t>
+          <t>Side-push tactile switch, SMD right angle, 4.7x2.3 mm</t>
         </is>
       </c>
     </row>
@@ -921,27 +921,27 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>TS-1010-C-A</t>
+          <t>MLT-5020</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Huaneng</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>C692458</t>
+          <t>C94598</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>SW1</t>
+          <t>BZ1</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Side-push tactile switch, SMD right angle, 4.7x2.3 mm</t>
+          <t>Magnetic buzzer, 4 kHz, 5x5 mm</t>
         </is>
       </c>
     </row>
@@ -951,27 +951,27 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>MLT-5020</t>
+          <t>SC-32S 32.768kHz 20PPM 12.5pF</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Huaneng</t>
+          <t>Seiko</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>C94598</t>
+          <t>C97606</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>BZ1</t>
+          <t>Y1</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Magnetic buzzer, 4 kHz, 5x5 mm</t>
+          <t>32.768 kHz crystal, 3215, 12.5 pF</t>
         </is>
       </c>
     </row>
@@ -981,27 +981,27 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>SC-32S 32.768kHz 20PPM 12.5pF</t>
+          <t>KT-0603R</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Seiko</t>
+          <t>Hubei KENTO</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>C97606</t>
+          <t>C2286</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Y1</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>32.768 kHz crystal, 3215, 12.5 pF</t>
+          <t>Red LED 0603 (Rec)</t>
         </is>
       </c>
     </row>
@@ -1011,27 +1011,27 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>KT-0603R</t>
+          <t>TJ-S1615SW6TGLCCYRGB-A5</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Hubei KENTO</t>
+          <t>TOGIALED</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>C2286</t>
+          <t>C273610</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Red LED 0603 (Rec)</t>
+          <t>RGB LED common anode, 1.6x1.5 mm (pin 1 anode; 2 B, 3 G, 4 R cathodes)</t>
         </is>
       </c>
     </row>
@@ -1041,127 +1041,127 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>TJ-S1615SW6TGLCCYRGB-A5</t>
+          <t>NCD0603G3</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>TOGIALED</t>
+          <t>NationStar</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>C273610</t>
+          <t>C7429914</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>RGB LED common anode, 1.6x1.5 mm (pin 1 anode; 2 B, 3 G, 4 R cathodes)</t>
+          <t>Green LED 0603 (charge)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>NCD0603G3</t>
+          <t>0402WGF5101TCE</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>NationStar</t>
+          <t>UNI-ROYAL</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>C7429914</t>
+          <t>C25905</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>R1,R2,R6</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Green LED 0603 (charge)</t>
+          <t>5.1k 1% 0402 (USB-C CC; charger PROG: 1000 V / 5.1k = 196 mA)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>0402WGF5101TCE</t>
+          <t>CL05A475KP5NRNC</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>UNI-ROYAL</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>C25905</t>
+          <t>C368809</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>R1,R2,R6</t>
+          <t>C1,C2</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>5.1k 1% 0402 (USB-C CC; charger PROG: 1000 V / 5.1k = 196 mA)</t>
+          <t>4.7 uF 10 V X5R 0402 (charger VDD and VBAT; MCP73831 needs at least 4.7 uF on each)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>CL05A475KP5NRNC</t>
+          <t>0402WGF1001TCE</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>UNI-ROYAL</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>C368809</t>
+          <t>C11702</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>C1,C2</t>
+          <t>R5,R7,R8</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>4.7 uF 10 V X5R 0402 (charger VDD and VBAT; MCP73831 needs at least 4.7 uF on each)</t>
+          <t>1k 1% 0402 (R5 BTN series ESD resistor; Rec LED; RGB red)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>0402WGF1001TCE</t>
+          <t>0402WGF5600TCE</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -1171,27 +1171,27 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>C11702</t>
+          <t>C25126</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>R5,R7,R8</t>
+          <t>R9,R10</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>1k 1% 0402 (R5 BTN series ESD resistor; Rec LED; RGB red)</t>
+          <t>560R 1% 0402 (RGB green, blue)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>0402WGF5600TCE</t>
+          <t>0402WGF2201TCE</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -1201,27 +1201,27 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>C25126</t>
+          <t>C25879</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>R9,R10</t>
+          <t>R3,R4,R11</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>560R 1% 0402 (RGB green, blue)</t>
+          <t>2.2k 1% 0402 (I2C pull-ups R3/R4: MAX17048 60 pF + 300 ns rise; charge LED R11)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>0402WGF2201TCE</t>
+          <t>0402WGF1003TCE</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -1231,27 +1231,27 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>C25879</t>
+          <t>C25741</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>R3,R4,R11</t>
+          <t>R12,R13,R15,R16,R17,R18,R20,R21</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2.2k 1% 0402 (I2C pull-ups R3/R4: MAX17048 60 pF + 300 ns rise; charge LED R11)</t>
+          <t>100k 1% 0402 (Q1, Q3-Q5 gate pull-downs; Q2 gate pull-up; U4 /CS pull-up; R20 Q7 gate to VBUS; R21 CHG_INHIBIT pull-down)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>0402WGF1003TCE</t>
+          <t>0402WGJ022JTCE</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1261,47 +1261,47 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>C25741</t>
+          <t>C25158</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>R12,R13,R15,R16,R17,R18,R20,R21</t>
+          <t>R14</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>100k 1% 0402 (Q1, Q3-Q5 gate pull-downs; Q2 gate pull-up; U4 /CS pull-up; R20 Q7 gate to VBUS; R21 CHG_INHIBIT pull-down)</t>
+          <t>2.2R 5% 0402 (U1 VBUS series, Nordic ref)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>0402WGJ022JTCE</t>
+          <t>CL05B104KO5NNNC</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>UNI-ROYAL</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>C25158</t>
+          <t>C1525</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>R14</t>
+          <t>C5,C10,C11,C13</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2.2R 5% 0402 (U1 VBUS series, Nordic ref)</t>
+          <t>100 nF 16 V X7R 0402 decoupling</t>
         </is>
       </c>
     </row>
@@ -1311,7 +1311,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>CL05B104KO5NNNC</t>
+          <t>CL05A105KA5NQNC</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -1321,27 +1321,27 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>C1525</t>
+          <t>C52923</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>C5,C10,C11,C13</t>
+          <t>C3,C4,C14,C15</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>100 nF 16 V X7R 0402 decoupling</t>
+          <t>1 uF 25 V X5R 0402 (U9 LDO in/out; U8 REG and VDD)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>CL05A105KA5NQNC</t>
+          <t>CL10A106KP8NNNC</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -1351,27 +1351,27 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>C52923</t>
+          <t>C19702</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>C3,C4,C14,C15</t>
+          <t>C6,C7,C12</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>1 uF 25 V X5R 0402 (U9 LDO in/out; U8 REG and VDD)</t>
+          <t>10 uF 10 V X5R 0603 (U1 VDD/VDDH and VBUS, Raytac ref 8.3; U7 accelerometer)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>CL10A106KP8NNNC</t>
+          <t>CL05C180JB5NNNC</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1381,17 +1381,17 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>C19702</t>
+          <t>C307443</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>C6,C7,C12</t>
+          <t>C8,C9</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>10 uF 10 V X5R 0603 (U1 VDD/VDDH and VBUS, Raytac ref 8.3; U7 accelerometer)</t>
+          <t>18 pF C0G 0402 (32.768 kHz load caps; checked against nRF52840 PS)</t>
         </is>
       </c>
     </row>
@@ -1401,87 +1401,87 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>CL05C180JB5NNNC</t>
+          <t>CC0402JRNPO9BN820</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>C307443</t>
+          <t>C107011</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>C8,C9</t>
+          <t>C16,C17</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>18 pF C0G 0402 (32.768 kHz load caps; checked against nRF52840 PS)</t>
+          <t>82 pF 5% NP0 50 V 0402 (NFC tuning for the Molex 146236-0101 antenna, 3.1 uH; Nordic nRF52840 PS p.461). Extended part: no Basic 82 pF 0402 exists.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>CC0402JRNPO9BN820</t>
+          <t>25121WF100JT4E</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>YAGEO</t>
+          <t>UNI-ROYAL</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>C107011</t>
+          <t>C47019</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>C16,C17</t>
+          <t>R19</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>82 pF 5% NP0 50 V 0402 (NFC tuning for the Molex 146236-0101 antenna, 3.1 uH; Nordic nRF52840 PS p.461). Extended part: no Basic 82 pF 0402 exists.</t>
+          <t>10R 1% 2512, 1 W (buzzer series resistor; survives a stuck-on Q1: 0.49 W)</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n">
+      <c r="A33" t="n">
         <v>1</v>
       </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>25121WF100JT4E</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>UNI-ROYAL</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>C47019</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>R19</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>10R 1% 2512, 1 W (buzzer series resistor; survives a stuck-on Q1: 0.49 W)</t>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>MDBT50Q-1MV2</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Raytac</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>C5118826</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>U1</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>nRF52840 module, chip antenna (pre-ordered at JLCPCB 8 Oct, held in My Parts)</t>
         </is>
       </c>
     </row>
@@ -1491,27 +1491,27 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>MDBT50Q-1MV2</t>
+          <t>SMD0805P050TF</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Raytac</t>
+          <t>RUILON</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>C5118826</t>
+          <t>C20978</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>nRF52840 module, chip antenna (pre-ordered at JLCPCB 8 Oct, held in My Parts)</t>
+          <t>Polyfuse 0.5 A hold / 1 A trip, 6 V, 0805 (battery rail; 0.33 A hold at 60 C)</t>
         </is>
       </c>
     </row>
@@ -1521,62 +1521,32 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>SMD0805P050TF</t>
+          <t>SMF5.0A</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>RUILON</t>
+          <t>MDD</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>C20978</t>
+          <t>C193402</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Polyfuse 0.5 A hold / 1 A trip, 6 V, 0805 (battery rail; 0.33 A hold at 60 C)</t>
+          <t>TVS 5 V standoff, 6.4-7 V breakdown, unidirectional, SOD-123FL (VBUS hot-plug; cathode to VBUS)</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="n">
-        <v>1</v>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>SMF5.0A</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>MDD</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>C193402</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>D5</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>TVS 5 V standoff, 6.4-7 V breakdown, unidirectional, SOD-123FL (VBUS hot-plug; cathode to VBUS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="3" t="inlineStr">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t>Quantities are per board. LCSC rounds up to each part's minimum order. Blank LCSC numbers: the BOM tool matches on the manufacturer part number.</t>
         </is>
@@ -2016,22 +1986,22 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>S2B-PH-SM4-TB(LF)(SN)</t>
+          <t>Battery wires (no connector)</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>C295747</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Verified</t>
+          <t>Not fitted</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>LCSC/JLC page: ~48-99k in stock.</t>
+          <t>No part. The JST PH side-entry header is 5.5 mm tall and would sit 0.8 mm above the case inside (PCB top 8.1 + 5.5 = 13.6 &gt; 12.8 mm). The battery leads are hand-soldered into two 0.5 mm holes (pad 1 = BATT_RAW +, pad 2 = GND -).</t>
         </is>
       </c>
     </row>
@@ -2739,7 +2709,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>500 mAh LiPo, 30 x 35 x 5.0 mm (+/-0.1), protection board (S-8261), JST-PH 2-pin with Adafruit polarity (pin 1 = +), 100 mm leads. Ground ship only. Check polarity with a meter before first plug-in.</t>
+          <t>500 mAh LiPo, 30 x 35 x 5.0 mm (+/-0.1), protection board (S-8261), 100 mm leads. Cut off the JST plug one wire at a time (never both together) and solder red to J2 + (pad 1), black to J2 - (pad 2). Ground ship only. Check polarity with a meter before soldering.</t>
         </is>
       </c>
     </row>
@@ -2786,7 +2756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3236,6 +3206,40 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>J2: JST PH S2B-PH-SM4-TB -&gt; 2 solder-wire holes (16 Oct)</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>The side-entry JST PH header is 5.5 mm tall; on the 1.0 mm board at its case height it would stand 0.8 mm into the case wall. Wires take no height.</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>J2 kept in the schematic (same nets) but excluded from BOM and placement files. Footprint Connector_Wire SolderWire-0.15sqmm 1x02 P4 mm, 0.5 mm holes, at the bottom-left near the battery lead end. Cut the battery plug off and solder red to + (pad 1), black to - (pad 2). Removed from the JLCPCB BOM (C295747).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>LED pins re-assigned (16 Oct)</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>The module pins run 25, 27, 29 left to right but the switches were R, G, B in the other order, so the blue line had to loop over the red and green escapes. Matching the order lets each LED line drop straight down.</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>U1 pin 25 (P1.08) -&gt; LED_R, pin 27 (P0.11) -&gt; LED_G, pin 29 (P0.12) -&gt; LED_B. All three are ordinary GPIOs driving FET gates. Firmware: use this pin map.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rev A order: Standard PCBA, 5 assembled; buy-elsewhere quantities for 5 units
- Fab README: Standard PCBA (U7 LIS2DW12 is Standard-only: LGA, X-ray),
  all 5 boards assembled.
- BOM Buy Elsewhere: motor, battery and NFC antenna at 6 each (5 units +
  1 spare); 24 M2 x 10 self-tapping screws added.
</commit_message>
<xml_diff>
--- a/Schematics/RevA/BOM/Jot_RevA_BOM.xlsx
+++ b/Schematics/RevA/BOM/Jot_RevA_BOM.xlsx
@@ -2610,7 +2610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2634,7 +2634,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Qty</t>
+          <t>Qty (5 units + 1 spare)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -2665,7 +2665,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
@@ -2695,7 +2695,7 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
@@ -2724,10 +2724,8 @@
           <t>Molex 146236-0101</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="C4" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
@@ -2742,6 +2740,36 @@
       <c r="F4" s="2" t="inlineStr">
         <is>
           <t>NFC flex antenna with ferrite, 15 x 25 mm + tab, 0.27 mm thick, 3.1 uH. Two fine wires from its pads to the AE1 holes. Solder quickly (thin polyimide tab).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>M2 x 10 self-tapping screws for plastic, head 4.0 mm across or less (the counterbore is 4.2 mm, 2.0 mm deep)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Amazon or McMaster-Carr</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>4 per unit: through the back shell and standoffs, PCB clamped, into the front bosses. 20 + 4 spare.</t>
         </is>
       </c>
     </row>

</xml_diff>